<commit_message>
Update mid-validation report and annexes
Revise Mid-Validation deliverables: updated ANFORA_Mid_Validation_Report_2026 (DOCX and PDF), refreshed ANFORA_Data_Collection_Mid_Validation.xlsx, and replaced annex PDFs (ENG & ESP) for Lucena coordination meeting, August 2026 outreach evidence, and Educator Webinar (2026-09-03).
</commit_message>
<xml_diff>
--- a/ANFORA_Data_Collection_Mid_Validation.xlsx
+++ b/ANFORA_Data_Collection_Mid_Validation.xlsx
@@ -183,7 +183,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -249,6 +249,8 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -576,12 +578,12 @@
           <t>D05 - ANFORA</t>
         </is>
       </c>
-      <c r="B2" s="15" t="n"/>
-      <c r="C2" s="15" t="n"/>
-      <c r="D2" s="16" t="n"/>
+      <c r="B2" s="23" t="n"/>
+      <c r="C2" s="23" t="n"/>
+      <c r="D2" s="24" t="n"/>
       <c r="E2" s="17" t="inlineStr">
         <is>
-          <t>March 1st - August 31st</t>
+          <t>1 March – 31 August 2026</t>
         </is>
       </c>
       <c r="F2" s="1" t="n"/>

</xml_diff>